<commit_message>
Add UK university mentions: alias table, YouTube suffix flag, TikTok + YT scrape
- Added 63 aliases for 11 UK universities to university_alias_table_v2.xlsx
  (official names, short names, hashtags: #bristoluniversity, #warwickuni etc.)
- Added --search-suffix flag to ingest_youtube.py (default: ' study australia',
  overrideable to ' study uk' for UK university searches)
- Ran TikTok hashtag scraper for all 11 UK unis: 1,905 rows ingested today
  (80-134 mentions per UK university)
- Ran YouTube scraper with ' study uk' suffix: 2 videos matched
- Ran aggregate.py — university_summary.csv now covers 11 UK + 10 AU unis

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mentions/university_alias_table_v2.xlsx
+++ b/mentions/university_alias_table_v2.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:F132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1505,7 +1505,6 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1629,7 +1628,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1657,7 +1655,6 @@
           <t>low</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1685,7 +1682,6 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1713,7 +1709,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1741,7 +1736,6 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1801,7 +1795,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1829,7 +1822,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1889,7 +1881,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1917,7 +1908,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1945,7 +1935,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1973,7 +1962,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2001,7 +1989,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2029,7 +2016,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2057,7 +2043,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2085,7 +2070,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2145,7 +2129,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2173,7 +2156,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2201,7 +2183,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2229,7 +2210,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2257,7 +2237,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2285,7 +2264,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2313,7 +2291,6 @@
           <t>high</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2341,7 +2318,1747 @@
           <t>high</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>University of Bristol</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>University of Bristol</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>University of Bristol</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Bristol University</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>University of Bristol</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Bristol</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>city name</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>University of Bristol</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>#BristolUniversity</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>University of Bristol</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>#bristoluni</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>University of Bristol</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>#studyatbristol</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>University of Bristol</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>#universityofbristol</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>University of Warwick</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>University of Warwick</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>University of Warwick</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Warwick University</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>University of Warwick</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Warwick</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>University of Warwick</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>#WarwickUniversity</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>University of Warwick</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>#warwickuni</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>University of Warwick</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>#studyatwarwick</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Durham University</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Durham University</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Durham University</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Durham</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>city name</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Durham University</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>#DurhamUniversity</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Durham University</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>#durhamuni</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Durham University</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>#studyatdurham</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>University of Bath</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>University of Bath</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>University of Bath</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Bath University</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>University of Bath</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Bath</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>city name</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>University of Bath</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>#BathUniversity</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>University of Bath</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>#bathuni</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>University of Bath</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>#studyatbath</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Newcastle University</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Newcastle University</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Newcastle University</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Newcastle</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>city name</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Newcastle University</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>NCL University</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>informal</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Newcastle University</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>#NewcastleUniversity</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Newcastle University</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>#newcastleuni</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Newcastle University</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>#studyatnewcastle</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>University of Exeter</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>University of Exeter</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>University of Exeter</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Exeter University</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>University of Exeter</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Exeter</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>University of Exeter</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>#ExeterUniversity</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>University of Exeter</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>#exeteruni</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>University of Exeter</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>#studyatexeter</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Lancaster University</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Lancaster University</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Lancaster University</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Lancaster</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>city name</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Lancaster University</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>#LancasterUniversity</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Lancaster University</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>#lancasteruni</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Lancaster University</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>#studyatlancaster</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>University of York</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>University of York</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>University of York</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>York University</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>University of York</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>York</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>city/collision risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>University of York</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>#YorkUniversity</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>University of York</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>#universityofyork</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>University of York</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>#studyatyork</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Cardiff University</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Cardiff University</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Cardiff University</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Cardiff</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>city name</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Cardiff University</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>#CardiffUniversity</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Cardiff University</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>#cardiffuni</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Cardiff University</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>#studyatcardiff</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Loughborough University</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Loughborough University</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Loughborough University</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Loughborough</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Loughborough University</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Lboro</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>informal</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Loughborough University</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>#LoughboroughUniversity</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Loughborough University</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>#loughboroughuni</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Loughborough University</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>#lborouni</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Swansea University</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Swansea University</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Swansea University</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Swansea</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>city name</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Swansea University</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>#SwanseaUniversity</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Swansea University</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>#swanseauni</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Swansea University</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>#studyatswansea</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>hashtag</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>